<commit_message>
Harden header encoding and template compatibility
</commit_message>
<xml_diff>
--- a/Raw data standard Title/FAKT 原始记录文件表头.xlsx
+++ b/Raw data standard Title/FAKT 原始记录文件表头.xlsx
@@ -56,34 +56,34 @@
     <t>Project run number</t>
   </si>
   <si>
-    <t>Temperature set point [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual value [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT1 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT2 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT3 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT4 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT5 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT6 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT7 [ｰC]</t>
-  </si>
-  <si>
-    <t>Temperature actual valueT8 [ｰC]</t>
+    <t>Temperature set point [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual value [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT1 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT2 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT3 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT4 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT5 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT6 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT7 [°C]</t>
+  </si>
+  <si>
+    <t>Temperature actual valueT8 [°C]</t>
   </si>
   <si>
     <t>Process air mass setpoint [kg/h]</t>
@@ -134,7 +134,7 @@
     <t>Temperature regulator LUT [kg/h]</t>
   </si>
   <si>
-    <t>Temperature regulator hold interval [ｰC]</t>
+    <t>Temperature regulator hold interval [°C]</t>
   </si>
   <si>
     <t>Temperature regulator output value [kg/h]</t>
@@ -176,52 +176,52 @@
     <t>Backpressure regulator outputvalue [%]</t>
   </si>
   <si>
-    <t>Tmp_ T1_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T1_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T2_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T2_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T3_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T3_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T4_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T4_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T5_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T5_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T6_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T6_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T7_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T7_max [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T8_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_ T8_max [ｰC]</t>
+    <t>Tmp_ T1_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T1_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T2_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T2_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T3_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T3_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T4_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T4_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T5_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T5_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T6_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T6_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T7_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T7_max [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T8_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_ T8_max [°C]</t>
   </si>
   <si>
     <t>Process air mass min [kg/h]</t>
@@ -251,10 +251,10 @@
     <t>Backpressure regulator mode</t>
   </si>
   <si>
-    <t>Tmp_min [ｰC]</t>
-  </si>
-  <si>
-    <t>Tmp_max [ｰC]</t>
+    <t>Tmp_min [°C]</t>
+  </si>
+  <si>
+    <t>Tmp_max [°C]</t>
   </si>
   <si>
     <t>Min/Max-Logger</t>
@@ -278,13 +278,13 @@
     <t>AI4</t>
   </si>
   <si>
-    <t>Transient TMP_i_1Hz [ｰK/s]</t>
-  </si>
-  <si>
-    <t>Transient TMP_i_10Hz [ｰK/s]</t>
-  </si>
-  <si>
-    <t>Transient TMP_i_100Hz [ｰK/s]</t>
+    <t>Transient TMP_i_1Hz [°K/s]</t>
+  </si>
+  <si>
+    <t>Transient TMP_i_10Hz [°K/s]</t>
+  </si>
+  <si>
+    <t>Transient TMP_i_100Hz [°K/s]</t>
   </si>
   <si>
     <t>Transient MPL_i_1Hz kg/h/s]</t>

</xml_diff>